<commit_message>
Plan v2 : 20 unites Coolbox propriete Havana (apport en nature 2,12 M$, 40 k$/unite/an), restauration et bars
</commit_message>
<xml_diff>
--- a/plan-affaires/Plan_affaires_Complexe_Havana_v2.xlsx
+++ b/plan-affaires/Plan_affaires_Complexe_Havana_v2.xlsx
@@ -2430,7 +2430,7 @@
         </is>
       </c>
       <c r="B2" s="4" t="n">
-        <v>2859800</v>
+        <v>3970000</v>
       </c>
     </row>
     <row r="3">
@@ -2440,7 +2440,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>235490</v>
+        <v>291000</v>
       </c>
     </row>
     <row r="4">
@@ -13194,22 +13194,22 @@
         <v>0.04</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>2058368.417371844</v>
+        <v>2011284.634760705</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>41167.36834743688</v>
+        <v>40225.69269521411</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>80688.04196097629</v>
+        <v>78842.35768261965</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>77460.52028253724</v>
+        <v>75688.66337531486</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>74362.09947123575</v>
+        <v>72661.11684030226</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>71387.61549238632</v>
+        <v>69754.67216669017</v>
       </c>
     </row>
     <row r="10">
@@ -13250,22 +13250,22 @@
         <v>0.1</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>1154744.682145605</v>
+        <v>2368846.347607053</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>57737.23410728024</v>
+        <v>118442.3173803526</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>109700.7448038325</v>
+        <v>225040.40302267</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>98730.6703234492</v>
+        <v>202536.362720403</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>88857.60329110429</v>
+        <v>182282.7264483627</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>79971.84296199385</v>
+        <v>164054.4538035264</v>
       </c>
     </row>
     <row r="12">
@@ -13278,22 +13278,22 @@
         <v>0.08</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>57176.90048255123</v>
+        <v>55869.01763224181</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>2287.076019302049</v>
+        <v>2234.760705289672</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>4391.185957059934</v>
+        <v>4290.740554156171</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>4039.89108049514</v>
+        <v>3947.481309823678</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>3716.699794055529</v>
+        <v>3631.682805037784</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>3419.363810531087</v>
+        <v>3341.148180634762</v>
       </c>
     </row>
     <row r="13">
@@ -14054,19 +14054,19 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>1.17</v>
+        <v>1.48</v>
       </c>
       <c r="C4" s="9" t="n">
-        <v>1.37</v>
+        <v>1.68</v>
       </c>
       <c r="D4" s="9" t="n">
-        <v>1.63</v>
+        <v>1.96</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>1.21</v>
+        <v>1.47</v>
       </c>
       <c r="F4" s="9" t="n">
-        <v>1.41</v>
+        <v>1.66</v>
       </c>
     </row>
     <row r="5">
@@ -14076,19 +14076,19 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.76</v>
+        <v>1.02</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>0.97</v>
+        <v>1.23</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>1.21</v>
+        <v>1.49</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>0.85</v>
+        <v>1.09</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>1.06</v>
+        <v>1.29</v>
       </c>
     </row>
     <row r="6">
@@ -14098,19 +14098,19 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.79</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>0.77</v>
+        <v>1.01</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>0.66</v>
+        <v>0.88</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>0.88</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="7">
@@ -14120,19 +14120,19 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>0.36</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="C7" s="9" t="n">
-        <v>0.57</v>
+        <v>0.78</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>0.79</v>
+        <v>1.02</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>0.47</v>
+        <v>0.66</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>0.68</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="8">
@@ -14142,19 +14142,19 @@
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>0.93</v>
+        <v>1.16</v>
       </c>
       <c r="C8" s="9" t="n">
-        <v>1.12</v>
+        <v>1.35</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>1.36</v>
+        <v>1.62</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>1</v>
+        <v>1.19</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>1.18</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="9">
@@ -14164,19 +14164,19 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.16</v>
       </c>
       <c r="C9" s="9" t="n">
-        <v>1.09</v>
+        <v>1.32</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>1.31</v>
+        <v>1.55</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>0.97</v>
+        <v>1.17</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>1.14</v>
+        <v>1.34</v>
       </c>
     </row>
     <row r="10">
@@ -14186,19 +14186,19 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>1.15</v>
+        <v>1.46</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>1.29</v>
+        <v>1.58</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>1.54</v>
+        <v>1.86</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>1.14</v>
+        <v>1.38</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>1.33</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="11">
@@ -14208,19 +14208,19 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>1.06</v>
+        <v>1.34</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>1.21</v>
+        <v>1.49</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>1.46</v>
+        <v>1.76</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>1.07</v>
+        <v>1.3</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>1.26</v>
+        <v>1.48</v>
       </c>
     </row>
     <row r="12">
@@ -14230,19 +14230,19 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>1.2</v>
+        <v>1.53</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>1.29</v>
+        <v>1.57</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>1.54</v>
+        <v>1.85</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>1.13</v>
+        <v>1.38</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>1.33</v>
+        <v>1.56</v>
       </c>
     </row>
     <row r="14">
@@ -14252,7 +14252,7 @@
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>0.4978529423306974</v>
+        <v>0.5141674560262713</v>
       </c>
     </row>
   </sheetData>

</xml_diff>